<commit_message>
Complete Literature Project Importer with Real LLM AI Screening
</commit_message>
<xml_diff>
--- a/samples/protocol.xlsx
+++ b/samples/protocol.xlsx
@@ -1,87 +1,135 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
-  <workbookPr filterPrivacy="true" defaultThemeVersion="164011"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28623"/>
+  <workbookPr defaultThemeVersion="166925"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ASUS\Dropbox\AI Tools\For Demo\2. SYMPRO\Archive\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{93C3FADD-D81D-469D-8E3C-51C007C84FC4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="14805" windowHeight="8010"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{72D25113-45C8-4524-A6F5-27B566310AA0}"/>
   </bookViews>
   <sheets>
-    <sheet name="Protocol" sheetId="1" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="122211"/>
+  <calcPr calcId="191028"/>
+  <extLst>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
+      <x15:workbookPr chartTrackingRefBase="1"/>
+    </ext>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="12">
-  <si>
-    <t>criterion1</t>
-  </si>
-  <si>
-    <t>criterion2</t>
-  </si>
-  <si>
-    <t>criterion3</t>
-  </si>
-  <si>
-    <t>criterion4</t>
-  </si>
-  <si>
-    <t>inclusion_criteria</t>
-  </si>
-  <si>
-    <t>exclusion_criteria</t>
-  </si>
-  <si>
-    <t>Randomized Controlled Trial (RCT) or Parallel-Group Clinical Trial design</t>
-  </si>
-  <si>
-    <t>Adults (aged 18+) diagnosed with Type 2 Diabetes Mellitus</t>
-  </si>
-  <si>
-    <t>Telemedicine, mobile health app, remote monitoring, or digital health intervention vs standard care</t>
-  </si>
-  <si>
-    <t>Reports primary quantitative glycemic outcomes (HbA1c reduction, time-in-range)</t>
-  </si>
-  <si>
-    <t>Primary original research RCTs published from 2018-2024 evaluating remote telemedicine or digital health interventions for adult Type 2 Diabetes patients with quantitative HbA1c outcomes.</t>
-  </si>
-  <si>
-    <t>Animal or in-vitro laboratory studies; pediatric populations (&lt;18 years); Type 1 Diabetes only; systematic reviews, meta-analyses, editorials, letters, commentaries, or conference abstracts lacking primary data.</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="22" uniqueCount="22">
+  <si>
+    <t>Population_Include</t>
+  </si>
+  <si>
+    <t>Population_Exclude</t>
+  </si>
+  <si>
+    <t>Intervention</t>
+  </si>
+  <si>
+    <t>Comparator</t>
+  </si>
+  <si>
+    <t>Clinical_Outcomes</t>
+  </si>
+  <si>
+    <t>Economic_Analysis_Outcomes</t>
+  </si>
+  <si>
+    <t>Treatment_Patterns_Outcomes</t>
+  </si>
+  <si>
+    <t>HRQoL_Outcomes</t>
+  </si>
+  <si>
+    <t>HRQoL_scales</t>
+  </si>
+  <si>
+    <t>Epidemiology_Outcomes</t>
+  </si>
+  <si>
+    <t>Economic_Burden_Outcomes</t>
+  </si>
+  <si>
+    <t>Other_Outcomes</t>
+  </si>
+  <si>
+    <t>Country_Check</t>
+  </si>
+  <si>
+    <t>StudyDesign_Include</t>
+  </si>
+  <si>
+    <t>StudyDesign_Exclude</t>
+  </si>
+  <si>
+    <t>HER2-positive Breast Cancer</t>
+  </si>
+  <si>
+    <t>Trastuzumab emtansine, T-DM1, trastuzumab deruxtecan, T-DXd</t>
+  </si>
+  <si>
+    <t>Efficacy outcome, ORR, CR, PR, OS, PFS, DFS, EFS, Safety outcome, AEs, discontinuation, Mortality/survival data</t>
+  </si>
+  <si>
+    <t>Clinical trials, RCT, Non-RCT, Observational studies, cross-sectional studies, cohort studies</t>
+  </si>
+  <si>
+    <t>Phase-I study, PK/PD studies</t>
+  </si>
+  <si>
+    <t>Other than HER2 positive Breast cancer
+HER2 negative breast cancer</t>
+  </si>
+  <si>
+    <t xml:space="preserve">EQ-5D (EQ-5D-3L / EQ-5D-5L) , EORTC QLQ-C30 , Other disease related or generic Patient reported outcomes (PROs) , Other disease related or generic health state utilities </t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:ap="http://schemas.openxmlformats.org/officeDocument/2006/extended-properties" xmlns:op="http://schemas.openxmlformats.org/officeDocument/2006/custom-properties" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cdr="http://schemas.openxmlformats.org/drawingml/2006/chartDrawing" xmlns:comp="http://schemas.openxmlformats.org/drawingml/2006/compatibility" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:lc="http://schemas.openxmlformats.org/drawingml/2006/lockedCanvas" xmlns:pic="http://schemas.openxmlformats.org/drawingml/2006/picture" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" xmlns:m="http://schemas.openxmlformats.org/officeDocument/2006/math" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:sl="http://schemas.openxmlformats.org/schemaLibrary/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xne="http://schemas.microsoft.com/office/excel/2006/main" xmlns:mso="http://schemas.microsoft.com/office/2006/01/customui" xmlns:ax="http://schemas.microsoft.com/office/2006/activeX" xmlns:cppr="http://schemas.microsoft.com/office/2006/coverPageProps" xmlns:cdip="http://schemas.microsoft.com/office/2006/customDocumentInformationPanel" xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ntns="http://schemas.microsoft.com/office/2006/metadata/customXsn" xmlns:lp="http://schemas.microsoft.com/office/2006/metadata/longProperties" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" xmlns:msink="http://schemas.microsoft.com/ink/2010/main" xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" xmlns:cdr14="http://schemas.microsoft.com/office/drawing/2010/chartDrawing" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" xmlns:pic14="http://schemas.microsoft.com/office/drawing/2010/picture" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xdr14="http://schemas.microsoft.com/office/excel/2010/spreadsheetDrawing" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:dsp="http://schemas.microsoft.com/office/drawing/2008/diagram" xmlns:mso14="http://schemas.microsoft.com/office/2009/07/customui" xmlns:dgm14="http://schemas.microsoft.com/office/drawing/2010/diagram" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x12ac="http://schemas.microsoft.com/office/spreadsheetml/2011/1/ac" xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xmlns:xr4="http://schemas.microsoft.com/office/spreadsheetml/2016/revision4" xmlns:xr5="http://schemas.microsoft.com/office/spreadsheetml/2016/revision5" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr7="http://schemas.microsoft.com/office/spreadsheetml/2016/revision7" xmlns:xr8="http://schemas.microsoft.com/office/spreadsheetml/2016/revision8" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr11="http://schemas.microsoft.com/office/spreadsheetml/2016/revision11" xmlns:xr12="http://schemas.microsoft.com/office/spreadsheetml/2016/revision12" xmlns:xr13="http://schemas.microsoft.com/office/spreadsheetml/2016/revision13" xmlns:xr14="http://schemas.microsoft.com/office/spreadsheetml/2016/revision14" xmlns:xr15="http://schemas.microsoft.com/office/spreadsheetml/2016/revision15" xmlns:x16="http://schemas.microsoft.com/office/spreadsheetml/2014/11/main" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:mo="http://schemas.microsoft.com/office/mac/office/2008/main" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:o="urn:schemas-microsoft-com:office:office" xmlns:v="urn:schemas-microsoft-com:vml" mc:Ignorable="c14 cdr14 a14 pic14 x14 xdr14 x14ac dsp mso14 dgm14 x15 x12ac x15ac xr xr2 xr3 xr4 xr5 xr6 xr7 xr8 xr9 xr10 xr11 xr12 xr13 xr14 xr15 x15 x16 x16r2 mo mx mv o v" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <fonts count="2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
-      <sz val="11"/>
+      <sz val="14"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
+      <scheme val="minor"/>
     </font>
     <font>
-      <b val="1"/>
-      <sz val="11"/>
-      <color rgb="FFFFFFFF"/>
+      <b/>
+      <sz val="14"/>
+      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="2">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FF059669"/>
-      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -96,22 +144,33 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="true" applyFill="true" applyAlignment="true">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
-  <tableStyles count="0" defaultPivotStyle="PivotStyleLight16" defaultTableStyle="TableStyleMedium2"/>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
     <a:clrScheme name="Office">
       <a:dk1>
@@ -127,7 +186,7 @@
         <a:srgbClr val="E7E6E6"/>
       </a:lt2>
       <a:accent1>
-        <a:srgbClr val="5B9BD5"/>
+        <a:srgbClr val="4472C4"/>
       </a:accent1>
       <a:accent2>
         <a:srgbClr val="ED7D31"/>
@@ -139,7 +198,7 @@
         <a:srgbClr val="FFC000"/>
       </a:accent4>
       <a:accent5>
-        <a:srgbClr val="4472C4"/>
+        <a:srgbClr val="5B9BD5"/>
       </a:accent5>
       <a:accent6>
         <a:srgbClr val="70AD47"/>
@@ -186,6 +245,23 @@
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
         <a:font script="Geor" typeface="Sylfaen"/>
+        <a:font script="Armn" typeface="Arial"/>
+        <a:font script="Bugi" typeface="Leelawadee UI"/>
+        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
+        <a:font script="Java" typeface="Javanese Text"/>
+        <a:font script="Lisu" typeface="Segoe UI"/>
+        <a:font script="Mymr" typeface="Myanmar Text"/>
+        <a:font script="Nkoo" typeface="Ebrima"/>
+        <a:font script="Olck" typeface="Nirmala UI"/>
+        <a:font script="Osma" typeface="Ebrima"/>
+        <a:font script="Phag" typeface="Phagspa"/>
+        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
+        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
+        <a:font script="Syre" typeface="Estrangelo Edessa"/>
+        <a:font script="Sora" typeface="Nirmala UI"/>
+        <a:font script="Tale" typeface="Microsoft Tai Le"/>
+        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
+        <a:font script="Tfng" typeface="Ebrima"/>
       </a:majorFont>
       <a:minorFont>
         <a:latin typeface="Calibri" panose="020F0502020204030204"/>
@@ -221,6 +297,23 @@
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
         <a:font script="Geor" typeface="Sylfaen"/>
+        <a:font script="Armn" typeface="Arial"/>
+        <a:font script="Bugi" typeface="Leelawadee UI"/>
+        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
+        <a:font script="Java" typeface="Javanese Text"/>
+        <a:font script="Lisu" typeface="Segoe UI"/>
+        <a:font script="Mymr" typeface="Myanmar Text"/>
+        <a:font script="Nkoo" typeface="Ebrima"/>
+        <a:font script="Olck" typeface="Nirmala UI"/>
+        <a:font script="Osma" typeface="Ebrima"/>
+        <a:font script="Phag" typeface="Phagspa"/>
+        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
+        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
+        <a:font script="Syre" typeface="Estrangelo Edessa"/>
+        <a:font script="Sora" typeface="Nirmala UI"/>
+        <a:font script="Tale" typeface="Microsoft Tai Le"/>
+        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
+        <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
     <a:fmtScheme name="Office">
@@ -363,60 +456,106 @@
   </a:themeElements>
   <a:objectDefaults/>
   <a:extraClrSchemeLst/>
+  <a:extLst>
+    <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+    </a:ext>
+  </a:extLst>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A86E2898-DE93-470E-8F36-FD5F85A7B8E1}">
+  <dimension ref="A1:O2"/>
+  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="25.2" customHeight="1" x14ac:dyDescent="0.35"/>
   <cols>
-    <col customWidth="true" max="2" min="1" width="25"/>
-    <col customWidth="true" max="3" min="3" width="30"/>
-    <col customWidth="true" max="4" min="4" width="28"/>
-    <col customWidth="true" max="6" min="5" width="45"/>
+    <col min="1" max="1" width="10.4140625" style="1" customWidth="1"/>
+    <col min="2" max="2" width="9.9140625" style="1" customWidth="1"/>
+    <col min="3" max="3" width="11.5" style="1" customWidth="1"/>
+    <col min="4" max="4" width="11.33203125" style="1" customWidth="1"/>
+    <col min="5" max="5" width="16" style="1" customWidth="1"/>
+    <col min="6" max="6" width="8.75" style="1" customWidth="1"/>
+    <col min="7" max="7" width="10.83203125" style="1" customWidth="1"/>
+    <col min="8" max="8" width="9.83203125" style="1" customWidth="1"/>
+    <col min="9" max="9" width="12.1640625" style="1" customWidth="1"/>
+    <col min="10" max="10" width="12.9140625" style="1" customWidth="1"/>
+    <col min="11" max="13" width="8.6640625" style="1"/>
+    <col min="14" max="14" width="11.4140625" style="1" customWidth="1"/>
+    <col min="15" max="15" width="11.33203125" style="1" customWidth="1"/>
+    <col min="16" max="16384" width="8.6640625" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" s="1" customFormat="true" ht="25" customHeight="true">
-      <c r="A1" s="1" t="s">
+    <row r="1" spans="1:15" s="2" customFormat="1" ht="64.2" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" s="2" t="s">
         <v>5</v>
       </c>
+      <c r="G1" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="J1" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="K1" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="L1" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="M1" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="N1" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="O1" s="2" t="s">
+        <v>14</v>
+      </c>
     </row>
-    <row r="2" ht="80" customHeight="true">
-      <c r="A2" t="s">
-        <v>6</v>
-      </c>
-      <c r="B2" t="s">
-        <v>7</v>
-      </c>
-      <c r="C2" t="s">
-        <v>8</v>
-      </c>
-      <c r="D2" t="s">
-        <v>9</v>
-      </c>
-      <c r="E2" t="s">
-        <v>10</v>
-      </c>
-      <c r="F2" t="s">
-        <v>11</v>
+    <row r="2" spans="1:15" ht="295.2" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A2" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="E2" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="H2" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="N2" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="O2" s="1" t="s">
+        <v>19</v>
       </c>
     </row>
   </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>